<commit_message>
SVN (res) commit #2306 by scriswellwsf       ruleset mods w/ cool roof updates for 2022 code (tic $1302)
</commit_message>
<xml_diff>
--- a/RulesetDev/Rulesets/CA Res/Rules/T24RClimateZoneCodeBaselines.xlsx
+++ b/RulesetDev/Rulesets/CA Res/Rules/T24RClimateZoneCodeBaselines.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\svn-CEC\SF_CBECC-Res\trunk\RulesetDev\Rulesets\CA Res\Rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4775BF9-BB3E-4266-B93D-1AF3E135781D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7575A7D-86F0-4C2C-B0FA-7186571AAF49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2490" windowWidth="20640" windowHeight="12015" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33600" yWindow="0" windowWidth="24060" windowHeight="14310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T24RClimateZoneCodeBaselines" sheetId="1" r:id="rId1"/>
@@ -3335,13 +3335,13 @@
     <t>AltLowRoofRiseAboveDeckIns - presriptive reqs for Altered, LowRoofRise (&lt; 2:12) roof above deck insulation</t>
   </si>
   <si>
-    <t>12/13/22 - SAC - added new col: AltLowRoofRiseAboveDeckIns - presriptive reqs for Altered, LowRoofRise (&lt; 2:12) roof above deck insulation (tic #1302)</t>
-  </si>
-  <si>
     <t>added - SAC 12/13/22 (tic #1302)</t>
   </si>
   <si>
     <t>R14 Sheathing</t>
+  </si>
+  <si>
+    <t>12/13/22 - SAC - added new col: AltLowRoofRiseAboveDeckIns - prescriptive reqs for Altered, LowRoofRise (&lt; 2:12) roof above deck insulation -and- revised SteepRoofReflect &amp; FlatRoofReflect for '22+ code vintages (tic #1302)</t>
   </si>
 </sst>
 </file>
@@ -4751,7 +4751,7 @@
         <v>2</v>
       </c>
       <c r="D5" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -5957,7 +5957,7 @@
         <v>339</v>
       </c>
       <c r="P101" s="12" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="Y101" t="s">
         <v>9</v>
@@ -52580,7 +52580,7 @@
         <v>116</v>
       </c>
       <c r="AU331" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV331" s="3" t="s">
         <v>116</v>
@@ -52803,7 +52803,7 @@
         <v>116</v>
       </c>
       <c r="AU332" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV332" s="3" t="s">
         <v>116</v>
@@ -53253,17 +53253,17 @@
       <c r="AQ334" s="27">
         <v>0</v>
       </c>
-      <c r="AR334" s="27">
-        <v>0.1</v>
-      </c>
-      <c r="AS334" s="27">
-        <v>0.1</v>
+      <c r="AR334" s="100">
+        <v>0.2</v>
+      </c>
+      <c r="AS334" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT334" s="3" t="s">
         <v>116</v>
       </c>
       <c r="AU334" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV334" s="3" t="s">
         <v>204</v>
@@ -53716,8 +53716,8 @@
       <c r="AR336" s="27">
         <v>0.1</v>
       </c>
-      <c r="AS336" s="27">
-        <v>0.1</v>
+      <c r="AS336" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT336" s="3" t="s">
         <v>116</v>
@@ -53945,8 +53945,8 @@
       <c r="AR337" s="27">
         <v>0.1</v>
       </c>
-      <c r="AS337" s="27">
-        <v>0.1</v>
+      <c r="AS337" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT337" s="3" t="s">
         <v>116</v>
@@ -54171,17 +54171,17 @@
       <c r="AQ338" s="27">
         <v>0</v>
       </c>
-      <c r="AR338" s="27">
-        <v>0.1</v>
-      </c>
-      <c r="AS338" s="27">
-        <v>0.1</v>
+      <c r="AR338" s="100">
+        <v>0.2</v>
+      </c>
+      <c r="AS338" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT338" s="3" t="s">
         <v>116</v>
       </c>
       <c r="AU338" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV338" s="3" t="s">
         <v>204</v>
@@ -54400,17 +54400,17 @@
       <c r="AQ339" s="27">
         <v>0</v>
       </c>
-      <c r="AR339" s="27">
-        <v>0.1</v>
-      </c>
-      <c r="AS339" s="27">
-        <v>0.1</v>
+      <c r="AR339" s="100">
+        <v>0.2</v>
+      </c>
+      <c r="AS339" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT339" s="3" t="s">
         <v>116</v>
       </c>
       <c r="AU339" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV339" s="3" t="s">
         <v>204</v>
@@ -54633,14 +54633,14 @@
       <c r="AR340" s="27">
         <v>0.2</v>
       </c>
-      <c r="AS340" s="27">
-        <v>0.1</v>
+      <c r="AS340" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT340" s="3" t="s">
         <v>116</v>
       </c>
       <c r="AU340" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV340" s="3" t="s">
         <v>204</v>
@@ -54863,14 +54863,14 @@
       <c r="AR341" s="27">
         <v>0.2</v>
       </c>
-      <c r="AS341" s="27">
-        <v>0.1</v>
+      <c r="AS341" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT341" s="3" t="s">
         <v>116</v>
       </c>
       <c r="AU341" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV341" s="3" t="s">
         <v>204</v>
@@ -55093,14 +55093,14 @@
       <c r="AR342" s="27">
         <v>0.2</v>
       </c>
-      <c r="AS342" s="27">
-        <v>0.1</v>
+      <c r="AS342" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT342" s="3" t="s">
         <v>116</v>
       </c>
       <c r="AU342" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV342" s="3" t="s">
         <v>204</v>
@@ -55330,7 +55330,7 @@
         <v>116</v>
       </c>
       <c r="AU343" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV343" s="3" t="s">
         <v>204</v>
@@ -55553,14 +55553,14 @@
       <c r="AR344" s="27">
         <v>0.2</v>
       </c>
-      <c r="AS344" s="27">
-        <v>0.1</v>
+      <c r="AS344" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT344" s="3" t="s">
         <v>116</v>
       </c>
       <c r="AU344" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV344" s="3" t="s">
         <v>204</v>
@@ -55790,7 +55790,7 @@
         <v>116</v>
       </c>
       <c r="AU345" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV345" s="3" t="s">
         <v>204</v>
@@ -56020,7 +56020,7 @@
         <v>116</v>
       </c>
       <c r="AU346" s="108" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV346" s="84" t="s">
         <v>204</v>
@@ -60236,7 +60236,7 @@
         <v>116</v>
       </c>
       <c r="AU364" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV364" s="3" t="s">
         <v>116</v>
@@ -60459,7 +60459,7 @@
         <v>116</v>
       </c>
       <c r="AU365" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV365" s="3" t="s">
         <v>116</v>
@@ -60909,17 +60909,17 @@
       <c r="AQ367" s="27">
         <v>0</v>
       </c>
-      <c r="AR367" s="27">
-        <v>0.1</v>
-      </c>
-      <c r="AS367" s="27">
-        <v>0.1</v>
+      <c r="AR367" s="100">
+        <v>0.2</v>
+      </c>
+      <c r="AS367" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT367" s="3" t="s">
         <v>116</v>
       </c>
       <c r="AU367" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV367" s="3" t="s">
         <v>204</v>
@@ -61372,8 +61372,8 @@
       <c r="AR369" s="27">
         <v>0.1</v>
       </c>
-      <c r="AS369" s="27">
-        <v>0.1</v>
+      <c r="AS369" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT369" s="3" t="s">
         <v>116</v>
@@ -61601,8 +61601,8 @@
       <c r="AR370" s="27">
         <v>0.1</v>
       </c>
-      <c r="AS370" s="27">
-        <v>0.1</v>
+      <c r="AS370" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT370" s="3" t="s">
         <v>116</v>
@@ -61827,17 +61827,17 @@
       <c r="AQ371" s="27">
         <v>0</v>
       </c>
-      <c r="AR371" s="27">
-        <v>0.1</v>
-      </c>
-      <c r="AS371" s="27">
-        <v>0.1</v>
+      <c r="AR371" s="100">
+        <v>0.2</v>
+      </c>
+      <c r="AS371" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT371" s="3" t="s">
         <v>116</v>
       </c>
       <c r="AU371" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV371" s="3" t="s">
         <v>204</v>
@@ -62056,17 +62056,17 @@
       <c r="AQ372" s="27">
         <v>0</v>
       </c>
-      <c r="AR372" s="27">
-        <v>0.1</v>
-      </c>
-      <c r="AS372" s="27">
-        <v>0.1</v>
+      <c r="AR372" s="100">
+        <v>0.2</v>
+      </c>
+      <c r="AS372" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT372" s="3" t="s">
         <v>116</v>
       </c>
       <c r="AU372" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV372" s="3" t="s">
         <v>204</v>
@@ -62289,14 +62289,14 @@
       <c r="AR373" s="27">
         <v>0.2</v>
       </c>
-      <c r="AS373" s="27">
-        <v>0.1</v>
+      <c r="AS373" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT373" s="3" t="s">
         <v>116</v>
       </c>
       <c r="AU373" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV373" s="3" t="s">
         <v>204</v>
@@ -62519,14 +62519,14 @@
       <c r="AR374" s="27">
         <v>0.2</v>
       </c>
-      <c r="AS374" s="27">
-        <v>0.1</v>
+      <c r="AS374" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT374" s="3" t="s">
         <v>116</v>
       </c>
       <c r="AU374" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV374" s="3" t="s">
         <v>204</v>
@@ -62749,14 +62749,14 @@
       <c r="AR375" s="27">
         <v>0.2</v>
       </c>
-      <c r="AS375" s="27">
-        <v>0.1</v>
+      <c r="AS375" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT375" s="3" t="s">
         <v>116</v>
       </c>
       <c r="AU375" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV375" s="3" t="s">
         <v>204</v>
@@ -62986,7 +62986,7 @@
         <v>116</v>
       </c>
       <c r="AU376" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV376" s="3" t="s">
         <v>204</v>
@@ -63209,14 +63209,14 @@
       <c r="AR377" s="27">
         <v>0.2</v>
       </c>
-      <c r="AS377" s="27">
-        <v>0.1</v>
+      <c r="AS377" s="100">
+        <v>0.63</v>
       </c>
       <c r="AT377" s="3" t="s">
         <v>116</v>
       </c>
       <c r="AU377" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV377" s="3" t="s">
         <v>204</v>
@@ -63446,7 +63446,7 @@
         <v>116</v>
       </c>
       <c r="AU378" s="99" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV378" s="3" t="s">
         <v>204</v>
@@ -63676,7 +63676,7 @@
         <v>116</v>
       </c>
       <c r="AU379" s="108" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AV379" s="84" t="s">
         <v>204</v>

</xml_diff>